<commit_message>
Refactor evaluation framework and add attack scoring prompts
- Updated `9_englishF1.py` to remove Excel file dependency and use DataFrame directly for F1 score computation.
- Introduced `model_metrics_common.py` to centralize dataset specifications and utility functions.
- Added new attack scoring prompts for both Chinese and English languages in `prompts.py`.
- Enhanced `pipeline.py` to support attack scoring with customizable maximum score.
- Modified request handling to utilize parsed scores when available.
- Updated tests to reflect changes in scoring logic and schema handling.
</commit_message>
<xml_diff>
--- a/data/9_new_chinesehatedata_model_f1_scores.xlsx
+++ b/data/9_new_chinesehatedata_model_f1_scores.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="16">
   <si>
     <t>model</t>
   </si>
@@ -31,7 +31,31 @@
     <t>f1</t>
   </si>
   <si>
-    <t>openai/gpt-5.1</t>
+    <t>baidu_ernie-4.5-21b-a3b</t>
+  </si>
+  <si>
+    <t>chatgpt5.1</t>
+  </si>
+  <si>
+    <t>claude4.5</t>
+  </si>
+  <si>
+    <t>deepseek_deepseek-r1-0528</t>
+  </si>
+  <si>
+    <t>deepseek_deepseek-v3.2-exp</t>
+  </si>
+  <si>
+    <t>meta-llama_llama-4-maverick</t>
+  </si>
+  <si>
+    <t>moonshotai_kimi-k2-thinking</t>
+  </si>
+  <si>
+    <t>qwen_qwen-2.5-72b-instruct</t>
+  </si>
+  <si>
+    <t>z-ai_glm-4.6</t>
   </si>
   <si>
     <t>cot</t>
@@ -395,7 +419,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -420,16 +444,16 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C2">
-        <v>0.7106518282988871</v>
+        <v>0.8095744680851064</v>
       </c>
       <c r="D2">
-        <v>0.745</v>
+        <v>0.6341666666666667</v>
       </c>
       <c r="E2">
-        <v>0.7274206672091131</v>
+        <v>0.711214953271028</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -437,16 +461,288 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3">
+        <v>0.8320180383314544</v>
+      </c>
+      <c r="D3">
+        <v>0.615</v>
+      </c>
+      <c r="E3">
+        <v>0.7072352659319597</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4">
+        <v>0.7740029542097489</v>
+      </c>
+      <c r="D4">
+        <v>0.4366666666666666</v>
+      </c>
+      <c r="E4">
+        <v>0.5583377730420884</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5">
+        <v>0.7908961593172119</v>
+      </c>
+      <c r="D5">
+        <v>0.4633333333333333</v>
+      </c>
+      <c r="E5">
+        <v>0.5843405149763531</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
         <v>7</v>
       </c>
-      <c r="C3">
-        <v>0.7905982905982906</v>
-      </c>
-      <c r="D3">
-        <v>0.4625</v>
-      </c>
-      <c r="E3">
-        <v>0.583596214511041</v>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6">
+        <v>0.7401490947816827</v>
+      </c>
+      <c r="D6">
+        <v>0.5791666666666667</v>
+      </c>
+      <c r="E6">
+        <v>0.6498363721365124</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7">
+        <v>0.7277992277992278</v>
+      </c>
+      <c r="D7">
+        <v>0.6283333333333333</v>
+      </c>
+      <c r="E7">
+        <v>0.6744186046511628</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8">
+        <v>0.7685393258426966</v>
+      </c>
+      <c r="D8">
+        <v>0.57</v>
+      </c>
+      <c r="E8">
+        <v>0.6545454545454545</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9">
+        <v>0.7675736961451247</v>
+      </c>
+      <c r="D9">
+        <v>0.5641666666666667</v>
+      </c>
+      <c r="E9">
+        <v>0.6503362151777138</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10">
+        <v>0.7961165048543689</v>
+      </c>
+      <c r="D10">
+        <v>0.4783333333333333</v>
+      </c>
+      <c r="E10">
+        <v>0.5976054138469548</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11">
+        <v>0.8026124818577649</v>
+      </c>
+      <c r="D11">
+        <v>0.4608333333333333</v>
+      </c>
+      <c r="E11">
+        <v>0.5854949708840657</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12">
+        <v>0.7160883280757098</v>
+      </c>
+      <c r="D12">
+        <v>0.7566666666666667</v>
+      </c>
+      <c r="E12">
+        <v>0.7358184764991896</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13">
+        <v>0.785024154589372</v>
+      </c>
+      <c r="D13">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="E13">
+        <v>0.6410256410256411</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14">
+        <v>0.7347222222222223</v>
+      </c>
+      <c r="D14">
+        <v>0.4408333333333334</v>
+      </c>
+      <c r="E14">
+        <v>0.5510416666666667</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15">
+        <v>0.7608695652173914</v>
+      </c>
+      <c r="D15">
+        <v>0.4958333333333333</v>
+      </c>
+      <c r="E15">
+        <v>0.6004036326942482</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16">
+        <v>0.7746144721233689</v>
+      </c>
+      <c r="D16">
+        <v>0.5441666666666667</v>
+      </c>
+      <c r="E16">
+        <v>0.6392559960841899</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17">
+        <v>0.7210727969348659</v>
+      </c>
+      <c r="D17">
+        <v>0.7841666666666667</v>
+      </c>
+      <c r="E17">
+        <v>0.7512974051896207</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18">
+        <v>0.7630813953488372</v>
+      </c>
+      <c r="D18">
+        <v>0.4375</v>
+      </c>
+      <c r="E18">
+        <v>0.5561440677966102</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B19" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19">
+        <v>0.7748776508972267</v>
+      </c>
+      <c r="D19">
+        <v>0.3958333333333333</v>
+      </c>
+      <c r="E19">
+        <v>0.5239933811362383</v>
       </c>
     </row>
   </sheetData>

</xml_diff>